<commit_message>
Rebuild: multi-asset reconciliation engine with scaled synthetic portfolio
</commit_message>
<xml_diff>
--- a/output/exception_report.xlsx
+++ b/output/exception_report.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
+      <color rgb="00595959"/>
       <sz val="11"/>
     </font>
     <font>
@@ -53,12 +54,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
@@ -66,13 +61,8 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -93,8 +83,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDF2F2"/>
-        <bgColor rgb="00FDF2F2"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2DCDB"/>
+        <bgColor rgb="00F2DCDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+        <bgColor rgb="00D6EAF8"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,7 +106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -126,16 +128,11 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
-    <border>
-      <bottom style="double">
-        <color rgb="001F497D"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,18 +140,40 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,32 +539,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INVESTMENT OPERATIONS RECONCILIATION REPORT</t>
+          <t>INVESTMENT OPERATIONS DAILY EXCEPTION REPORT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As-Of Date: 2026-07-15</t>
+          <t>As-Of Date: 2026-07-24 | Source: Reconciliation Engine v2</t>
         </is>
       </c>
     </row>
@@ -557,213 +578,627 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>URGENT ESCALATIONS REQUIRED</t>
+          <t>TOTAL CAPITAL AT RISK ($)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>2</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1361714.799999992</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>PART A: CASH LINE-ITEM RECONCILIATION</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Security ID</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Security Name</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Asset Class</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Qty (Internal)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Qty (Custodian)</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Qty Variance</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>MV (Internal)</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>MV (Custodian)</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>MV Variance</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Exception Type</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Security ID</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Qty (Internal)</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Qty (Custodian)</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Qty Variance</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>MV (Internal)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>MV (Custodian)</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>MV Variance</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Exception Classification</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>ALT_INF_MEL</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>MEL_AIRPORT</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Melbourne Airport Infrastructure Fund</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Unlisted/Alternatives</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>4169739</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>3810307.33</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>359431.6699999999</v>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>UNLISTED_VALUATION_LAG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>CASH001</t>
+          <t>ALT_PE_COLLINS</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D9" s="8" t="n">
+          <t>COLLINS_PE</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Collins St Private Equity Fund III</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Unlisted/Alternatives</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>2387076</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>2183729.77</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>203346.23</v>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>UNLISTED_VALUATION_LAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>AU_EQ_CBA</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>CBA</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Commonwealth Bank of Australia</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>AU Equities</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>5890</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>5845</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>2394991.8</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>2376693.9</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>18297.89999999991</v>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>CA_DRP_TIMING_LAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>AU_EQ_TLS</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Telstra Group</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>AU Equities</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>8822</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>8285</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>537</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>229460.22</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>215492.85</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>13967.37</v>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>QUANTITY_BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>AU_EQ_WES</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>WES</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Wesfarmers Ltd</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>AU Equities</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>4926</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>4431</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>495</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>1284208.2</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>1155161.7</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>129046.5</v>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>QUANTITY_BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>CASH_AUD</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>CASH_AUD</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Cash - Australian Dollar</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>764685</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>716185</v>
+      </c>
+      <c r="H13" s="11" t="n">
         <v>48500</v>
       </c>
-      <c r="E9" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G9" s="9" t="n">
+      <c r="I13" s="12" t="n">
+        <v>764685</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>716185</v>
+      </c>
+      <c r="K13" s="12" t="n">
         <v>48500</v>
       </c>
-      <c r="H9" s="9" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>Cash Balance Break</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>PART B: SECURITIES &amp; HOLDINGS RECONCILIATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Security ID</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Qty (Internal)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Qty (Custodian)</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Qty Variance</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>MV (Internal)</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>MV (Custodian)</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>MV Variance</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Exception Classification</t>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>CASH_BALANCE_BREAK</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>UNLISTED_INF01</t>
+          <t>FI_CORP_TLS</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>MEL_AIRPORT</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E14" s="8" t="n">
+          <t>CTLS28</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Telstra Corporate Bond 2028</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Fixed Income</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>2273415</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>2273415</v>
+      </c>
+      <c r="H14" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="9" t="n">
-        <v>1250000</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>Unlisted Asset Valuation Lag (Stale Custody Price Certificate)</t>
+      <c r="I14" s="9" t="n">
+        <v>231433647</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>230970779.71</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>462867.2899999917</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>COUPON_TIMING_LAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>US_EQ_AAPL</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>US Equities</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>9166</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>9166</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v>3137888.44</v>
+      </c>
+      <c r="J15" s="15" t="n">
+        <v>3155407.47</v>
+      </c>
+      <c r="K15" s="15" t="n">
+        <v>-17519.03000000026</v>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>FX_VALUATION_BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>US_EQ_JPM</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>US Equities</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>2028</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>2028</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>80815.8</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>79010.88</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>1804.919999999998</v>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>PRICING_BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>US_EQ_META</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Meta Platforms Inc.</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>US Equities</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>8234</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>8234</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>4454841.02</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>4348787.1</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>106053.9199999999</v>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>PRICING_BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>US_EQ_NVDA</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>NVIDIA Corp.</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>US Equities</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>3247</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>3247</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v>685117</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <v>685996.97</v>
+      </c>
+      <c r="K18" s="15" t="n">
+        <v>-879.9699999999721</v>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>FX_VALUATION_BREAK</t>
         </is>
       </c>
     </row>

</xml_diff>